<commit_message>
feat(marketing): implement SEO growth and release foundations
</commit_message>
<xml_diff>
--- a/docs/assets/downloads/templates/ffe-schedule.xlsx
+++ b/docs/assets/downloads/templates/ffe-schedule.xlsx
@@ -32,7 +32,7 @@
     <t>How to use</t>
   </si>
   <si>
-    <t>Agree the classification boundary with your team. In this library, furniture and the loose rug sit in this register; the retained floor belongs in the finish schedule and built-in joinery stays linked to its drawing and specification. This is a documentation convention, not a universal accounting rule.</t>
+    <t>Agree the classification boundary with your team. In this library, furniture and the loose rug sit in this register; the retained floor belongs in the finish schedule and built-in joinery stays linked to its drawing and specification. This is a documentation convention, not a universal accounting rule. Reconcile each stable reference against the plan once, then check its specification and purchasing unit before sharing.</t>
   </si>
   <si>
     <t>Example status</t>
@@ -653,7 +653,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="2" ht="76" customHeight="1" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="2" ht="92" customHeight="1" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A2" s="3" t="s">
         <v>2</v>
       </c>

</xml_diff>

<commit_message>
fix(marketing): close release QA gaps and publish accessible walkthroughs
</commit_message>
<xml_diff>
--- a/docs/assets/downloads/templates/ffe-schedule.xlsx
+++ b/docs/assets/downloads/templates/ffe-schedule.xlsx
@@ -1140,7 +1140,7 @@
   <sheetPr>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:I25"/>
+  <dimension ref="A1:I8"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="3" width="27" customWidth="1"/>
@@ -1317,206 +1317,16 @@
         <v>54</v>
       </c>
     </row>
-    <row r="9" ht="36" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A9" s="8"/>
-      <c r="B9" s="8"/>
-      <c r="C9" s="8"/>
-      <c r="D9" s="8"/>
-      <c r="E9" s="8"/>
-      <c r="F9" s="8"/>
-      <c r="G9" s="8"/>
-      <c r="H9" s="8"/>
-      <c r="I9" s="8"/>
-    </row>
-    <row r="10" ht="36" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A10" s="7"/>
-      <c r="B10" s="7"/>
-      <c r="C10" s="7"/>
-      <c r="D10" s="7"/>
-      <c r="E10" s="7"/>
-      <c r="F10" s="7"/>
-      <c r="G10" s="7"/>
-      <c r="H10" s="7"/>
-      <c r="I10" s="7"/>
-    </row>
-    <row r="11" ht="36" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A11" s="8"/>
-      <c r="B11" s="8"/>
-      <c r="C11" s="8"/>
-      <c r="D11" s="8"/>
-      <c r="E11" s="8"/>
-      <c r="F11" s="8"/>
-      <c r="G11" s="8"/>
-      <c r="H11" s="8"/>
-      <c r="I11" s="8"/>
-    </row>
-    <row r="12" ht="36" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A12" s="7"/>
-      <c r="B12" s="7"/>
-      <c r="C12" s="7"/>
-      <c r="D12" s="7"/>
-      <c r="E12" s="7"/>
-      <c r="F12" s="7"/>
-      <c r="G12" s="7"/>
-      <c r="H12" s="7"/>
-      <c r="I12" s="7"/>
-    </row>
-    <row r="13" ht="36" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A13" s="8"/>
-      <c r="B13" s="8"/>
-      <c r="C13" s="8"/>
-      <c r="D13" s="8"/>
-      <c r="E13" s="8"/>
-      <c r="F13" s="8"/>
-      <c r="G13" s="8"/>
-      <c r="H13" s="8"/>
-      <c r="I13" s="8"/>
-    </row>
-    <row r="14" ht="36" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A14" s="7"/>
-      <c r="B14" s="7"/>
-      <c r="C14" s="7"/>
-      <c r="D14" s="7"/>
-      <c r="E14" s="7"/>
-      <c r="F14" s="7"/>
-      <c r="G14" s="7"/>
-      <c r="H14" s="7"/>
-      <c r="I14" s="7"/>
-    </row>
-    <row r="15" ht="36" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A15" s="8"/>
-      <c r="B15" s="8"/>
-      <c r="C15" s="8"/>
-      <c r="D15" s="8"/>
-      <c r="E15" s="8"/>
-      <c r="F15" s="8"/>
-      <c r="G15" s="8"/>
-      <c r="H15" s="8"/>
-      <c r="I15" s="8"/>
-    </row>
-    <row r="16" ht="36" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A16" s="7"/>
-      <c r="B16" s="7"/>
-      <c r="C16" s="7"/>
-      <c r="D16" s="7"/>
-      <c r="E16" s="7"/>
-      <c r="F16" s="7"/>
-      <c r="G16" s="7"/>
-      <c r="H16" s="7"/>
-      <c r="I16" s="7"/>
-    </row>
-    <row r="17" ht="36" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A17" s="8"/>
-      <c r="B17" s="8"/>
-      <c r="C17" s="8"/>
-      <c r="D17" s="8"/>
-      <c r="E17" s="8"/>
-      <c r="F17" s="8"/>
-      <c r="G17" s="8"/>
-      <c r="H17" s="8"/>
-      <c r="I17" s="8"/>
-    </row>
-    <row r="18" ht="36" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A18" s="7"/>
-      <c r="B18" s="7"/>
-      <c r="C18" s="7"/>
-      <c r="D18" s="7"/>
-      <c r="E18" s="7"/>
-      <c r="F18" s="7"/>
-      <c r="G18" s="7"/>
-      <c r="H18" s="7"/>
-      <c r="I18" s="7"/>
-    </row>
-    <row r="19" ht="36" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A19" s="8"/>
-      <c r="B19" s="8"/>
-      <c r="C19" s="8"/>
-      <c r="D19" s="8"/>
-      <c r="E19" s="8"/>
-      <c r="F19" s="8"/>
-      <c r="G19" s="8"/>
-      <c r="H19" s="8"/>
-      <c r="I19" s="8"/>
-    </row>
-    <row r="20" ht="36" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A20" s="7"/>
-      <c r="B20" s="7"/>
-      <c r="C20" s="7"/>
-      <c r="D20" s="7"/>
-      <c r="E20" s="7"/>
-      <c r="F20" s="7"/>
-      <c r="G20" s="7"/>
-      <c r="H20" s="7"/>
-      <c r="I20" s="7"/>
-    </row>
-    <row r="21" ht="36" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A21" s="8"/>
-      <c r="B21" s="8"/>
-      <c r="C21" s="8"/>
-      <c r="D21" s="8"/>
-      <c r="E21" s="8"/>
-      <c r="F21" s="8"/>
-      <c r="G21" s="8"/>
-      <c r="H21" s="8"/>
-      <c r="I21" s="8"/>
-    </row>
-    <row r="22" ht="36" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A22" s="7"/>
-      <c r="B22" s="7"/>
-      <c r="C22" s="7"/>
-      <c r="D22" s="7"/>
-      <c r="E22" s="7"/>
-      <c r="F22" s="7"/>
-      <c r="G22" s="7"/>
-      <c r="H22" s="7"/>
-      <c r="I22" s="7"/>
-    </row>
-    <row r="23" ht="36" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A23" s="8"/>
-      <c r="B23" s="8"/>
-      <c r="C23" s="8"/>
-      <c r="D23" s="8"/>
-      <c r="E23" s="8"/>
-      <c r="F23" s="8"/>
-      <c r="G23" s="8"/>
-      <c r="H23" s="8"/>
-      <c r="I23" s="8"/>
-    </row>
-    <row r="24" ht="36" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A24" s="7"/>
-      <c r="B24" s="7"/>
-      <c r="C24" s="7"/>
-      <c r="D24" s="7"/>
-      <c r="E24" s="7"/>
-      <c r="F24" s="7"/>
-      <c r="G24" s="7"/>
-      <c r="H24" s="7"/>
-      <c r="I24" s="7"/>
-    </row>
-    <row r="25" ht="36" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A25" s="8"/>
-      <c r="B25" s="8"/>
-      <c r="C25" s="8"/>
-      <c r="D25" s="8"/>
-      <c r="E25" s="8"/>
-      <c r="F25" s="8"/>
-      <c r="G25" s="8"/>
-      <c r="H25" s="8"/>
-      <c r="I25" s="8"/>
-    </row>
   </sheetData>
-  <autoFilter ref="A5:I25"/>
+  <autoFilter ref="A5:I8"/>
   <mergeCells count="4">
     <mergeCell ref="A1:I1"/>
     <mergeCell ref="A2:I2"/>
     <mergeCell ref="A3:I3"/>
     <mergeCell ref="A4:I4"/>
   </mergeCells>
-  <dataValidations count="2">
-    <dataValidation type="decimal" operator="greaterThanOrEqual" allowBlank="1" showErrorMessage="1" errorStyle="stop" errorTitle="Use a non-negative number" error="Enter zero or a positive number, or leave unresolved inputs blank." sqref="D10:D25">
-      <formula1>0</formula1>
-    </dataValidation>
-    <dataValidation type="decimal" operator="greaterThanOrEqual" allowBlank="1" showErrorMessage="1" errorStyle="stop" errorTitle="Use a non-negative number" error="Enter zero or a positive number, or leave unresolved inputs blank." sqref="D6:D25">
+  <dataValidations count="1">
+    <dataValidation type="decimal" operator="greaterThanOrEqual" allowBlank="1" showErrorMessage="1" errorStyle="stop" errorTitle="Use a non-negative number" error="Enter zero or a positive number, or leave unresolved inputs blank." sqref="D6:D8">
       <formula1>0</formula1>
     </dataValidation>
   </dataValidations>

</xml_diff>

<commit_message>
feat(seo): implement audited resources and studio outcome reporting
</commit_message>
<xml_diff>
--- a/docs/assets/downloads/templates/ffe-schedule.xlsx
+++ b/docs/assets/downloads/templates/ffe-schedule.xlsx
@@ -9,7 +9,7 @@
     <sheet sheetId="3" name="Worked Example" state="visible" r:id="rId6"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm.Print_Area" localSheetId="0">'Instructions'!$A1:$B18</definedName>
+    <definedName name="_xlnm.Print_Area" localSheetId="0">'Instructions'!$A1:$B20</definedName>
     <definedName name="_xlnm.Print_Titles" localSheetId="0">'Instructions'!$1:$1</definedName>
     <definedName name="_xlnm.Print_Area" localSheetId="1">'Blank Template'!$A1:$I25</definedName>
     <definedName name="_xlnm.Print_Titles" localSheetId="1">'Blank Template'!$1:$5</definedName>
@@ -21,7 +21,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="86" uniqueCount="55">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="90" uniqueCount="59">
   <si>
     <t>FF&amp;E schedule template</t>
   </si>
@@ -57,6 +57,18 @@
   </si>
   <si>
     <t>These are educational planning aids, not legal agreements, professional certification, or instructions for construction.</t>
+  </si>
+  <si>
+    <t>Google Sheets import</t>
+  </si>
+  <si>
+    <t>Upload the XLSX to your own Drive and open it in Google Sheets. Before using it, check formulas, blank-versus-zero behavior, validation, number formats and print breaks. Keep the original XLSX. This workbook has not been independently checked in Google Sheets.</t>
+  </si>
+  <si>
+    <t>Printing</t>
+  </si>
+  <si>
+    <t>US Letter, landscape. Fit one page wide and inspect the preview; long tables may span multiple pages.</t>
   </si>
   <si>
     <t>Step 1</t>
@@ -272,26 +284,32 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="11">
+  <cellXfs count="13">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment vertical="top" wrapText="1"/>
+      <alignment horizontal="left" vertical="top" wrapText="1" indent="1"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment vertical="top" wrapText="1"/>
+      <alignment horizontal="left" vertical="top" wrapText="1" indent="1"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment vertical="top" wrapText="1"/>
+      <alignment horizontal="left" vertical="top" wrapText="1" indent="1"/>
     </xf>
     <xf numFmtId="0" fontId="6" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment vertical="top" wrapText="1"/>
+      <alignment horizontal="left" vertical="top" wrapText="1" indent="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="3" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1" indent="1"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
@@ -638,7 +656,7 @@
   <sheetPr>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:B18"/>
+  <dimension ref="A1:B20"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="30" customWidth="1"/>
@@ -693,7 +711,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="7" ht="48" customHeight="1" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="7" ht="60" customHeight="1" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A7" s="3" t="s">
         <v>12</v>
       </c>
@@ -789,8 +807,24 @@
         <v>35</v>
       </c>
     </row>
+    <row r="19" ht="48" customHeight="1" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A19" s="3" t="s">
+        <v>36</v>
+      </c>
+      <c r="B19" s="3" t="s">
+        <v>37</v>
+      </c>
+    </row>
+    <row r="20" ht="48" customHeight="1" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A20" s="3" t="s">
+        <v>38</v>
+      </c>
+      <c r="B20" s="3" t="s">
+        <v>39</v>
+      </c>
+    </row>
   </sheetData>
-  <pageSetup paperSize="9" orientation="landscape" fitToWidth="1" fitToHeight="0"/>
+  <pageSetup paperSize="1" orientation="landscape" fitToWidth="1" fitToHeight="0"/>
   <headerFooter>
     <oddFooter>&amp;LOpenLintel | Instructions &amp;RPage &amp;P</oddFooter>
   </headerFooter>
@@ -805,10 +839,12 @@
   <dimension ref="A1:I25"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
-    <col min="1" max="3" width="27" customWidth="1"/>
-    <col min="4" max="4" width="18" customWidth="1"/>
-    <col min="5" max="8" width="27" customWidth="1"/>
-    <col min="9" max="9" width="48" customWidth="1"/>
+    <col min="1" max="1" width="15" customWidth="1"/>
+    <col min="2" max="2" width="12" customWidth="1"/>
+    <col min="3" max="3" width="20" customWidth="1"/>
+    <col min="5" max="5" width="7" customWidth="1"/>
+    <col min="6" max="8" width="15" customWidth="1"/>
+    <col min="9" max="9" width="26" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" ht="32" customHeight="1" spans="1:9" s="4" customFormat="1" x14ac:dyDescent="0.25">
@@ -826,7 +862,7 @@
     </row>
     <row r="2" ht="38" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A2" s="3" t="s">
-        <v>36</v>
+        <v>40</v>
       </c>
       <c r="B2" s="3"/>
       <c r="C2" s="3"/>
@@ -839,7 +875,7 @@
     </row>
     <row r="3" ht="26" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A3" s="3" t="s">
-        <v>37</v>
+        <v>41</v>
       </c>
       <c r="B3" s="3"/>
       <c r="C3" s="3"/>
@@ -852,7 +888,7 @@
     </row>
     <row r="4" ht="28" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A4" s="3" t="s">
-        <v>38</v>
+        <v>42</v>
       </c>
       <c r="B4" s="3"/>
       <c r="C4" s="3"/>
@@ -865,31 +901,31 @@
     </row>
     <row r="5" ht="38" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A5" s="6" t="s">
-        <v>18</v>
+        <v>22</v>
       </c>
       <c r="B5" s="6" t="s">
-        <v>20</v>
+        <v>24</v>
       </c>
       <c r="C5" s="6" t="s">
-        <v>22</v>
+        <v>26</v>
       </c>
       <c r="D5" s="6" t="s">
-        <v>24</v>
+        <v>28</v>
       </c>
       <c r="E5" s="6" t="s">
-        <v>26</v>
+        <v>30</v>
       </c>
       <c r="F5" s="6" t="s">
-        <v>28</v>
+        <v>32</v>
       </c>
       <c r="G5" s="6" t="s">
-        <v>30</v>
+        <v>34</v>
       </c>
       <c r="H5" s="6" t="s">
-        <v>32</v>
+        <v>36</v>
       </c>
       <c r="I5" s="6" t="s">
-        <v>34</v>
+        <v>38</v>
       </c>
     </row>
     <row r="6" ht="36" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
@@ -1128,7 +1164,8 @@
       <formula1>0</formula1>
     </dataValidation>
   </dataValidations>
-  <pageSetup paperSize="9" orientation="landscape" fitToWidth="1" fitToHeight="0"/>
+  <pageMargins left="0.4" right="0.4" top="0.45" bottom="0.45" header="0.2" footer="0.2"/>
+  <pageSetup paperSize="1" orientation="landscape" fitToWidth="1" fitToHeight="0"/>
   <headerFooter>
     <oddFooter>&amp;LOpenLintel | Educational planning resource &amp;RPage &amp;P</oddFooter>
   </headerFooter>
@@ -1143,10 +1180,12 @@
   <dimension ref="A1:I8"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
-    <col min="1" max="3" width="27" customWidth="1"/>
-    <col min="4" max="4" width="18" customWidth="1"/>
-    <col min="5" max="8" width="27" customWidth="1"/>
-    <col min="9" max="9" width="48" customWidth="1"/>
+    <col min="1" max="1" width="15" customWidth="1"/>
+    <col min="2" max="2" width="12" customWidth="1"/>
+    <col min="3" max="3" width="20" customWidth="1"/>
+    <col min="5" max="5" width="7" customWidth="1"/>
+    <col min="6" max="8" width="15" customWidth="1"/>
+    <col min="9" max="9" width="26" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" ht="32" customHeight="1" spans="1:9" s="4" customFormat="1" x14ac:dyDescent="0.25">
@@ -1177,7 +1216,7 @@
     </row>
     <row r="3" ht="26" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A3" s="3" t="s">
-        <v>37</v>
+        <v>41</v>
       </c>
       <c r="B3" s="3"/>
       <c r="C3" s="3"/>
@@ -1190,7 +1229,7 @@
     </row>
     <row r="4" ht="28" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A4" s="3" t="s">
-        <v>38</v>
+        <v>42</v>
       </c>
       <c r="B4" s="3"/>
       <c r="C4" s="3"/>
@@ -1203,118 +1242,118 @@
     </row>
     <row r="5" ht="38" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A5" s="6" t="s">
-        <v>18</v>
+        <v>22</v>
       </c>
       <c r="B5" s="6" t="s">
-        <v>20</v>
+        <v>24</v>
       </c>
       <c r="C5" s="6" t="s">
-        <v>22</v>
+        <v>26</v>
       </c>
       <c r="D5" s="6" t="s">
-        <v>24</v>
+        <v>28</v>
       </c>
       <c r="E5" s="6" t="s">
-        <v>26</v>
+        <v>30</v>
       </c>
       <c r="F5" s="6" t="s">
-        <v>28</v>
+        <v>32</v>
       </c>
       <c r="G5" s="6" t="s">
-        <v>30</v>
+        <v>34</v>
       </c>
       <c r="H5" s="6" t="s">
-        <v>32</v>
+        <v>36</v>
       </c>
       <c r="I5" s="6" t="s">
-        <v>34</v>
-      </c>
-    </row>
-    <row r="6" ht="80" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
+        <v>38</v>
+      </c>
+    </row>
+    <row r="6" ht="72" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A6" s="9" t="s">
-        <v>39</v>
+        <v>43</v>
       </c>
       <c r="B6" s="9" t="s">
-        <v>40</v>
+        <v>44</v>
       </c>
       <c r="C6" s="9" t="s">
-        <v>41</v>
-      </c>
-      <c r="D6" s="9">
+        <v>45</v>
+      </c>
+      <c r="D6" s="10">
         <v>1</v>
       </c>
       <c r="E6" s="9" t="s">
-        <v>42</v>
+        <v>46</v>
       </c>
       <c r="F6" s="9" t="s">
+        <v>47</v>
+      </c>
+      <c r="G6" s="9" t="s">
+        <v>48</v>
+      </c>
+      <c r="H6" s="9" t="s">
+        <v>49</v>
+      </c>
+      <c r="I6" s="9" t="s">
+        <v>50</v>
+      </c>
+    </row>
+    <row r="7" ht="72" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A7" s="11" t="s">
         <v>43</v>
       </c>
-      <c r="G6" s="9" t="s">
-        <v>44</v>
-      </c>
-      <c r="H6" s="9" t="s">
-        <v>45</v>
-      </c>
-      <c r="I6" s="9" t="s">
+      <c r="B7" s="11" t="s">
+        <v>51</v>
+      </c>
+      <c r="C7" s="11" t="s">
+        <v>52</v>
+      </c>
+      <c r="D7" s="12">
+        <v>1</v>
+      </c>
+      <c r="E7" s="11" t="s">
         <v>46</v>
       </c>
-    </row>
-    <row r="7" ht="80" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A7" s="10" t="s">
-        <v>39</v>
-      </c>
-      <c r="B7" s="10" t="s">
-        <v>47</v>
-      </c>
-      <c r="C7" s="10" t="s">
+      <c r="F7" s="11" t="s">
+        <v>53</v>
+      </c>
+      <c r="G7" s="11" t="s">
         <v>48</v>
       </c>
-      <c r="D7" s="10">
+      <c r="H7" s="11" t="s">
+        <v>49</v>
+      </c>
+      <c r="I7" s="11" t="s">
+        <v>54</v>
+      </c>
+    </row>
+    <row r="8" ht="72" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A8" s="9" t="s">
+        <v>43</v>
+      </c>
+      <c r="B8" s="9" t="s">
+        <v>55</v>
+      </c>
+      <c r="C8" s="9" t="s">
+        <v>56</v>
+      </c>
+      <c r="D8" s="10">
         <v>1</v>
       </c>
-      <c r="E7" s="10" t="s">
-        <v>42</v>
-      </c>
-      <c r="F7" s="10" t="s">
+      <c r="E8" s="9" t="s">
+        <v>46</v>
+      </c>
+      <c r="F8" s="9" t="s">
+        <v>57</v>
+      </c>
+      <c r="G8" s="9" t="s">
+        <v>48</v>
+      </c>
+      <c r="H8" s="9" t="s">
         <v>49</v>
       </c>
-      <c r="G7" s="10" t="s">
-        <v>44</v>
-      </c>
-      <c r="H7" s="10" t="s">
-        <v>45</v>
-      </c>
-      <c r="I7" s="10" t="s">
-        <v>50</v>
-      </c>
-    </row>
-    <row r="8" ht="80" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A8" s="9" t="s">
-        <v>39</v>
-      </c>
-      <c r="B8" s="9" t="s">
-        <v>51</v>
-      </c>
-      <c r="C8" s="9" t="s">
-        <v>52</v>
-      </c>
-      <c r="D8" s="9">
-        <v>1</v>
-      </c>
-      <c r="E8" s="9" t="s">
-        <v>42</v>
-      </c>
-      <c r="F8" s="9" t="s">
-        <v>53</v>
-      </c>
-      <c r="G8" s="9" t="s">
-        <v>44</v>
-      </c>
-      <c r="H8" s="9" t="s">
-        <v>45</v>
-      </c>
       <c r="I8" s="9" t="s">
-        <v>54</v>
+        <v>58</v>
       </c>
     </row>
   </sheetData>
@@ -1330,7 +1369,8 @@
       <formula1>0</formula1>
     </dataValidation>
   </dataValidations>
-  <pageSetup paperSize="9" orientation="landscape" fitToWidth="1" fitToHeight="0"/>
+  <pageMargins left="0.4" right="0.4" top="0.45" bottom="0.45" header="0.2" footer="0.2"/>
+  <pageSetup paperSize="1" orientation="landscape" fitToWidth="1" fitToHeight="0"/>
   <headerFooter>
     <oddFooter>&amp;LOpenLintel | Educational planning resource &amp;RPage &amp;P</oddFooter>
   </headerFooter>

</xml_diff>

<commit_message>
feat(seo): implement audited resources and studio outcome reporting (#24)
Co-authored-by: Workspace <workspace@m13943.contaboserver.net>
</commit_message>
<xml_diff>
--- a/docs/assets/downloads/templates/ffe-schedule.xlsx
+++ b/docs/assets/downloads/templates/ffe-schedule.xlsx
@@ -9,7 +9,7 @@
     <sheet sheetId="3" name="Worked Example" state="visible" r:id="rId6"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm.Print_Area" localSheetId="0">'Instructions'!$A1:$B18</definedName>
+    <definedName name="_xlnm.Print_Area" localSheetId="0">'Instructions'!$A1:$B20</definedName>
     <definedName name="_xlnm.Print_Titles" localSheetId="0">'Instructions'!$1:$1</definedName>
     <definedName name="_xlnm.Print_Area" localSheetId="1">'Blank Template'!$A1:$I25</definedName>
     <definedName name="_xlnm.Print_Titles" localSheetId="1">'Blank Template'!$1:$5</definedName>
@@ -21,7 +21,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="86" uniqueCount="55">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="90" uniqueCount="59">
   <si>
     <t>FF&amp;E schedule template</t>
   </si>
@@ -57,6 +57,18 @@
   </si>
   <si>
     <t>These are educational planning aids, not legal agreements, professional certification, or instructions for construction.</t>
+  </si>
+  <si>
+    <t>Google Sheets import</t>
+  </si>
+  <si>
+    <t>Upload the XLSX to your own Drive and open it in Google Sheets. Before using it, check formulas, blank-versus-zero behavior, validation, number formats and print breaks. Keep the original XLSX. This workbook has not been independently checked in Google Sheets.</t>
+  </si>
+  <si>
+    <t>Printing</t>
+  </si>
+  <si>
+    <t>US Letter, landscape. Fit one page wide and inspect the preview; long tables may span multiple pages.</t>
   </si>
   <si>
     <t>Step 1</t>
@@ -272,26 +284,32 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="11">
+  <cellXfs count="13">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment vertical="top" wrapText="1"/>
+      <alignment horizontal="left" vertical="top" wrapText="1" indent="1"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment vertical="top" wrapText="1"/>
+      <alignment horizontal="left" vertical="top" wrapText="1" indent="1"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment vertical="top" wrapText="1"/>
+      <alignment horizontal="left" vertical="top" wrapText="1" indent="1"/>
     </xf>
     <xf numFmtId="0" fontId="6" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment vertical="top" wrapText="1"/>
+      <alignment horizontal="left" vertical="top" wrapText="1" indent="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="3" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1" indent="1"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
@@ -638,7 +656,7 @@
   <sheetPr>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:B18"/>
+  <dimension ref="A1:B20"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="30" customWidth="1"/>
@@ -693,7 +711,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="7" ht="48" customHeight="1" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="7" ht="60" customHeight="1" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A7" s="3" t="s">
         <v>12</v>
       </c>
@@ -789,8 +807,24 @@
         <v>35</v>
       </c>
     </row>
+    <row r="19" ht="48" customHeight="1" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A19" s="3" t="s">
+        <v>36</v>
+      </c>
+      <c r="B19" s="3" t="s">
+        <v>37</v>
+      </c>
+    </row>
+    <row r="20" ht="48" customHeight="1" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A20" s="3" t="s">
+        <v>38</v>
+      </c>
+      <c r="B20" s="3" t="s">
+        <v>39</v>
+      </c>
+    </row>
   </sheetData>
-  <pageSetup paperSize="9" orientation="landscape" fitToWidth="1" fitToHeight="0"/>
+  <pageSetup paperSize="1" orientation="landscape" fitToWidth="1" fitToHeight="0"/>
   <headerFooter>
     <oddFooter>&amp;LOpenLintel | Instructions &amp;RPage &amp;P</oddFooter>
   </headerFooter>
@@ -805,10 +839,12 @@
   <dimension ref="A1:I25"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
-    <col min="1" max="3" width="27" customWidth="1"/>
-    <col min="4" max="4" width="18" customWidth="1"/>
-    <col min="5" max="8" width="27" customWidth="1"/>
-    <col min="9" max="9" width="48" customWidth="1"/>
+    <col min="1" max="1" width="15" customWidth="1"/>
+    <col min="2" max="2" width="12" customWidth="1"/>
+    <col min="3" max="3" width="20" customWidth="1"/>
+    <col min="5" max="5" width="7" customWidth="1"/>
+    <col min="6" max="8" width="15" customWidth="1"/>
+    <col min="9" max="9" width="26" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" ht="32" customHeight="1" spans="1:9" s="4" customFormat="1" x14ac:dyDescent="0.25">
@@ -826,7 +862,7 @@
     </row>
     <row r="2" ht="38" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A2" s="3" t="s">
-        <v>36</v>
+        <v>40</v>
       </c>
       <c r="B2" s="3"/>
       <c r="C2" s="3"/>
@@ -839,7 +875,7 @@
     </row>
     <row r="3" ht="26" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A3" s="3" t="s">
-        <v>37</v>
+        <v>41</v>
       </c>
       <c r="B3" s="3"/>
       <c r="C3" s="3"/>
@@ -852,7 +888,7 @@
     </row>
     <row r="4" ht="28" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A4" s="3" t="s">
-        <v>38</v>
+        <v>42</v>
       </c>
       <c r="B4" s="3"/>
       <c r="C4" s="3"/>
@@ -865,31 +901,31 @@
     </row>
     <row r="5" ht="38" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A5" s="6" t="s">
-        <v>18</v>
+        <v>22</v>
       </c>
       <c r="B5" s="6" t="s">
-        <v>20</v>
+        <v>24</v>
       </c>
       <c r="C5" s="6" t="s">
-        <v>22</v>
+        <v>26</v>
       </c>
       <c r="D5" s="6" t="s">
-        <v>24</v>
+        <v>28</v>
       </c>
       <c r="E5" s="6" t="s">
-        <v>26</v>
+        <v>30</v>
       </c>
       <c r="F5" s="6" t="s">
-        <v>28</v>
+        <v>32</v>
       </c>
       <c r="G5" s="6" t="s">
-        <v>30</v>
+        <v>34</v>
       </c>
       <c r="H5" s="6" t="s">
-        <v>32</v>
+        <v>36</v>
       </c>
       <c r="I5" s="6" t="s">
-        <v>34</v>
+        <v>38</v>
       </c>
     </row>
     <row r="6" ht="36" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
@@ -1128,7 +1164,8 @@
       <formula1>0</formula1>
     </dataValidation>
   </dataValidations>
-  <pageSetup paperSize="9" orientation="landscape" fitToWidth="1" fitToHeight="0"/>
+  <pageMargins left="0.4" right="0.4" top="0.45" bottom="0.45" header="0.2" footer="0.2"/>
+  <pageSetup paperSize="1" orientation="landscape" fitToWidth="1" fitToHeight="0"/>
   <headerFooter>
     <oddFooter>&amp;LOpenLintel | Educational planning resource &amp;RPage &amp;P</oddFooter>
   </headerFooter>
@@ -1143,10 +1180,12 @@
   <dimension ref="A1:I8"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
-    <col min="1" max="3" width="27" customWidth="1"/>
-    <col min="4" max="4" width="18" customWidth="1"/>
-    <col min="5" max="8" width="27" customWidth="1"/>
-    <col min="9" max="9" width="48" customWidth="1"/>
+    <col min="1" max="1" width="15" customWidth="1"/>
+    <col min="2" max="2" width="12" customWidth="1"/>
+    <col min="3" max="3" width="20" customWidth="1"/>
+    <col min="5" max="5" width="7" customWidth="1"/>
+    <col min="6" max="8" width="15" customWidth="1"/>
+    <col min="9" max="9" width="26" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" ht="32" customHeight="1" spans="1:9" s="4" customFormat="1" x14ac:dyDescent="0.25">
@@ -1177,7 +1216,7 @@
     </row>
     <row r="3" ht="26" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A3" s="3" t="s">
-        <v>37</v>
+        <v>41</v>
       </c>
       <c r="B3" s="3"/>
       <c r="C3" s="3"/>
@@ -1190,7 +1229,7 @@
     </row>
     <row r="4" ht="28" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A4" s="3" t="s">
-        <v>38</v>
+        <v>42</v>
       </c>
       <c r="B4" s="3"/>
       <c r="C4" s="3"/>
@@ -1203,118 +1242,118 @@
     </row>
     <row r="5" ht="38" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A5" s="6" t="s">
-        <v>18</v>
+        <v>22</v>
       </c>
       <c r="B5" s="6" t="s">
-        <v>20</v>
+        <v>24</v>
       </c>
       <c r="C5" s="6" t="s">
-        <v>22</v>
+        <v>26</v>
       </c>
       <c r="D5" s="6" t="s">
-        <v>24</v>
+        <v>28</v>
       </c>
       <c r="E5" s="6" t="s">
-        <v>26</v>
+        <v>30</v>
       </c>
       <c r="F5" s="6" t="s">
-        <v>28</v>
+        <v>32</v>
       </c>
       <c r="G5" s="6" t="s">
-        <v>30</v>
+        <v>34</v>
       </c>
       <c r="H5" s="6" t="s">
-        <v>32</v>
+        <v>36</v>
       </c>
       <c r="I5" s="6" t="s">
-        <v>34</v>
-      </c>
-    </row>
-    <row r="6" ht="80" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
+        <v>38</v>
+      </c>
+    </row>
+    <row r="6" ht="72" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A6" s="9" t="s">
-        <v>39</v>
+        <v>43</v>
       </c>
       <c r="B6" s="9" t="s">
-        <v>40</v>
+        <v>44</v>
       </c>
       <c r="C6" s="9" t="s">
-        <v>41</v>
-      </c>
-      <c r="D6" s="9">
+        <v>45</v>
+      </c>
+      <c r="D6" s="10">
         <v>1</v>
       </c>
       <c r="E6" s="9" t="s">
-        <v>42</v>
+        <v>46</v>
       </c>
       <c r="F6" s="9" t="s">
+        <v>47</v>
+      </c>
+      <c r="G6" s="9" t="s">
+        <v>48</v>
+      </c>
+      <c r="H6" s="9" t="s">
+        <v>49</v>
+      </c>
+      <c r="I6" s="9" t="s">
+        <v>50</v>
+      </c>
+    </row>
+    <row r="7" ht="72" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A7" s="11" t="s">
         <v>43</v>
       </c>
-      <c r="G6" s="9" t="s">
-        <v>44</v>
-      </c>
-      <c r="H6" s="9" t="s">
-        <v>45</v>
-      </c>
-      <c r="I6" s="9" t="s">
+      <c r="B7" s="11" t="s">
+        <v>51</v>
+      </c>
+      <c r="C7" s="11" t="s">
+        <v>52</v>
+      </c>
+      <c r="D7" s="12">
+        <v>1</v>
+      </c>
+      <c r="E7" s="11" t="s">
         <v>46</v>
       </c>
-    </row>
-    <row r="7" ht="80" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A7" s="10" t="s">
-        <v>39</v>
-      </c>
-      <c r="B7" s="10" t="s">
-        <v>47</v>
-      </c>
-      <c r="C7" s="10" t="s">
+      <c r="F7" s="11" t="s">
+        <v>53</v>
+      </c>
+      <c r="G7" s="11" t="s">
         <v>48</v>
       </c>
-      <c r="D7" s="10">
+      <c r="H7" s="11" t="s">
+        <v>49</v>
+      </c>
+      <c r="I7" s="11" t="s">
+        <v>54</v>
+      </c>
+    </row>
+    <row r="8" ht="72" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A8" s="9" t="s">
+        <v>43</v>
+      </c>
+      <c r="B8" s="9" t="s">
+        <v>55</v>
+      </c>
+      <c r="C8" s="9" t="s">
+        <v>56</v>
+      </c>
+      <c r="D8" s="10">
         <v>1</v>
       </c>
-      <c r="E7" s="10" t="s">
-        <v>42</v>
-      </c>
-      <c r="F7" s="10" t="s">
+      <c r="E8" s="9" t="s">
+        <v>46</v>
+      </c>
+      <c r="F8" s="9" t="s">
+        <v>57</v>
+      </c>
+      <c r="G8" s="9" t="s">
+        <v>48</v>
+      </c>
+      <c r="H8" s="9" t="s">
         <v>49</v>
       </c>
-      <c r="G7" s="10" t="s">
-        <v>44</v>
-      </c>
-      <c r="H7" s="10" t="s">
-        <v>45</v>
-      </c>
-      <c r="I7" s="10" t="s">
-        <v>50</v>
-      </c>
-    </row>
-    <row r="8" ht="80" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A8" s="9" t="s">
-        <v>39</v>
-      </c>
-      <c r="B8" s="9" t="s">
-        <v>51</v>
-      </c>
-      <c r="C8" s="9" t="s">
-        <v>52</v>
-      </c>
-      <c r="D8" s="9">
-        <v>1</v>
-      </c>
-      <c r="E8" s="9" t="s">
-        <v>42</v>
-      </c>
-      <c r="F8" s="9" t="s">
-        <v>53</v>
-      </c>
-      <c r="G8" s="9" t="s">
-        <v>44</v>
-      </c>
-      <c r="H8" s="9" t="s">
-        <v>45</v>
-      </c>
       <c r="I8" s="9" t="s">
-        <v>54</v>
+        <v>58</v>
       </c>
     </row>
   </sheetData>
@@ -1330,7 +1369,8 @@
       <formula1>0</formula1>
     </dataValidation>
   </dataValidations>
-  <pageSetup paperSize="9" orientation="landscape" fitToWidth="1" fitToHeight="0"/>
+  <pageMargins left="0.4" right="0.4" top="0.45" bottom="0.45" header="0.2" footer="0.2"/>
+  <pageSetup paperSize="1" orientation="landscape" fitToWidth="1" fitToHeight="0"/>
   <headerFooter>
     <oddFooter>&amp;LOpenLintel | Educational planning resource &amp;RPage &amp;P</oddFooter>
   </headerFooter>

</xml_diff>